<commit_message>
feat: Auto-create user on bulk import surat tugas
</commit_message>
<xml_diff>
--- a/public/templates/surat_tugas_import_template.xlsx
+++ b/public/templates/surat_tugas_import_template.xlsx
@@ -15,7 +15,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
+  <si>
+    <t>nama_petugas</t>
+  </si>
   <si>
     <t>email_petugas</t>
   </si>
@@ -26,6 +29,9 @@
     <t>tempat_tugas</t>
   </si>
   <si>
+    <t>Andi</t>
+  </si>
+  <si>
     <t>andi@bps.go.id</t>
   </si>
   <si>
@@ -33,6 +39,9 @@
   </si>
   <si>
     <t>Kecamatan Demak</t>
+  </si>
+  <si>
+    <t>Budi</t>
   </si>
   <si>
     <t>budi@bps.go.id</t>
@@ -381,15 +390,16 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="25.851" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="25.851" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -399,27 +409,36 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>